<commit_message>
On-prem MPO: 9/17 refresh -- Fever Tree, Carbliss, HUSA exports + Promos_Report_26
Fever Tree 20 -> 21 (Robin Feldman, Courtyard Wayne tonic), Carbliss
17 -> 20 (Allison Scott +2, Brian Sengebush +1), HUSA holds at 1,
Bardstown menu 10 -> 15 (Brian Sengebush 0 -> 5 at Krogh's -- one
brand submitted twice, flagged in README). Report_26's four Yave rows
filtered out on merge; archive 11 -> 16 rows. Hub reads the new JSON
with no code change.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EUWjRSBHzvPcf8WiDRWa9t
</commit_message>
<xml_diff>
--- a/MPOs/on-prem/bardstown_menu_promos.xlsx
+++ b/MPOs/on-prem/bardstown_menu_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:11 PM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,45 +601,39 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
@@ -648,10 +642,14 @@
         </is>
       </c>
       <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -668,55 +666,49 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
@@ -725,10 +717,14 @@
         </is>
       </c>
       <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -745,17 +741,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 05:28 PM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -777,22 +773,22 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M4" s="2" t="n"/>
@@ -820,67 +816,65 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:08 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n"/>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="n"/>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -897,67 +891,65 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:01 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="n"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -974,12 +966,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1012,22 +1004,22 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M7" s="2" t="n"/>
@@ -1051,65 +1043,67 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:53 AM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK TAV (A)</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>31027</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>250 PARK AVE</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent, Menu</t>
-        </is>
-      </c>
+      <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1126,7 +1120,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:51 AM</t>
+          <t>09/15/2026 05:28 PM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1136,7 +1130,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1152,25 +1146,23 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>RED BULL VENDING MACHINE</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>120001</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>150 WAGARAW RD</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
@@ -1179,10 +1171,14 @@
         </is>
       </c>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="n"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1199,65 +1195,67 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 04:48 PM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>15004</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>1145 MCBRIDE AVE</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>STANHOPE</t>
         </is>
       </c>
       <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1274,33 +1272,37 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
+          <t>Feature Activation</t>
         </is>
       </c>
       <c r="H11" s="2" t="n">
@@ -1308,37 +1310,29 @@
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>HILTON HASBRK HTS #50591</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>34018</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>650 TERRACE AVE</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>HASBROUCK HEIGHTS</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="inlineStr">
-        <is>
-          <t>Drink Special</t>
-        </is>
-      </c>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent</t>
-        </is>
-      </c>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n"/>
+      <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1355,33 +1349,37 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
+          <t>Feature Activation</t>
         </is>
       </c>
       <c r="H12" s="2" t="n">
@@ -1389,45 +1387,422 @@
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="n"/>
+      <c r="N12" s="2" t="n"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2026 08:53 AM</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Nicholas Melissari</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>NEW PARK TAV (A)</t>
+        </is>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>31027</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>250 PARK AVE</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>EAST RUTHERFORD</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="n"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent, Menu</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2026 08:51 AM</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Nicholas Melissari</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="n"/>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>RED BULL VENDING MACHINE</t>
+        </is>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>120001</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>150 WAGARAW RD</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="n"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q14" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>09/09/2026 04:48 PM</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>allison scott</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>1145 MCBRIDE AVE</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>WOODLAND PARK</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q15" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n"/>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
           <t>HILTON HASBRK HTS #50591</t>
         </is>
       </c>
-      <c r="J12" s="2" t="inlineStr">
+      <c r="J16" s="2" t="inlineStr">
         <is>
           <t>34018</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr">
+      <c r="K16" s="2" t="inlineStr">
         <is>
           <t>650 TERRACE AVE</t>
         </is>
       </c>
-      <c r="L12" s="2" t="inlineStr">
+      <c r="L16" s="2" t="inlineStr">
         <is>
           <t>HASBROUCK HEIGHTS</t>
         </is>
       </c>
-      <c r="M12" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
         <is>
           <t>Drink Special</t>
         </is>
       </c>
-      <c r="N12" s="2" t="inlineStr">
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>Table Tent</t>
         </is>
       </c>
-      <c r="O12" s="2" t="inlineStr">
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q16" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n"/>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>HILTON HASBRK HTS #50591</t>
+        </is>
+      </c>
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>34018</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>650 TERRACE AVE</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>HASBROUCK HEIGHTS</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Drink Special</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COLLAB SERIES GOOSE ISLAND</t>
         </is>
       </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="P17" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COMPANY</t>
         </is>
       </c>
-      <c r="Q12" s="3" t="inlineStr">
+      <c r="Q17" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -1446,6 +1821,11 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q11" r:id="rId10"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId16"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
MPO refresh 2026-09-25: on-prem RDE exports + Promos_Report_33, off-prem cooler doors from Promos_Report_32
On-prem September: Fever Tree 21 -> 23, Carbliss 50 -> 69 (Paul Mclaughlin
joins Robin Feldman at goal), HUSA 1 -> 2 (Allison Scott's first draft
line), Bardstown 15 -> 16 (Adam Badalamenti, Hudson Farm Club). Robin
Feldman's Il Villaggio Carbliss row left the export and drops.

Off-prem September: Promos_Report_32 is the cooler door wrap pull -- 15 new
stickers, 60 -> 73 distinct, Phil Ernst 0 -> 12 (new at goal). RDE
datasets rebuilt byte-identical from the 9/23 exports.

The hub reads both boards' data at runtime, so it picks these up with no
change of its own.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RoV2mL1CCfk1vAYF2Fe2nK
</commit_message>
<xml_diff>
--- a/MPOs/on-prem/bardstown_menu_promos.xlsx
+++ b/MPOs/on-prem/bardstown_menu_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q17"/>
+  <dimension ref="A1:Q18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:11 PM</t>
+          <t>09/24/2026 03:54 PM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -612,44 +612,46 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>HUDSON FARM CLUB</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>230126</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>270 STANHOPE SPARTA RD</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>ANDOVER</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -666,12 +668,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/16/2026 02:11 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -724,7 +726,7 @@
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -746,7 +748,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -799,7 +801,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -816,12 +818,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:08 PM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -874,7 +876,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -891,12 +893,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:01 PM</t>
+          <t>09/16/2026 02:08 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -949,7 +951,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -966,55 +968,49 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:01 PM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
@@ -1023,10 +1019,14 @@
         </is>
       </c>
       <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="n"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1103,7 +1103,7 @@
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1120,65 +1120,67 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 05:28 PM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1195,67 +1197,65 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/15/2026 05:28 PM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="n"/>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>HAWTHORNE</t>
         </is>
       </c>
       <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="n"/>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1277,7 +1277,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1354,7 +1354,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1409,7 +1409,7 @@
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1426,62 +1426,64 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:53 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK TAV (A)</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>31027</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>250 PARK AVE</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>STANHOPE</t>
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent, Menu</t>
-        </is>
-      </c>
+      <c r="N13" s="2" t="n"/>
       <c r="O13" s="2" t="inlineStr">
         <is>
           <t>GREEN RIVER HONEY FINISHED BOURBON</t>
@@ -1501,12 +1503,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:51 AM</t>
+          <t>09/11/2026 08:53 AM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1527,34 +1529,36 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>RED BULL VENDING MACHINE</t>
+          <t>NEW PARK TAV (A)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>120001</t>
+          <t>31027</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>150 WAGARAW RD</t>
+          <t>250 PARK AVE</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>EAST RUTHERFORD</t>
         </is>
       </c>
       <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="n"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent, Menu</t>
+        </is>
+      </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
           <t>GREEN RIVER HONEY FINISHED BOURBON</t>
@@ -1574,7 +1578,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 04:48 PM</t>
+          <t>09/11/2026 08:51 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
@@ -1584,7 +1588,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1600,39 +1604,37 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+          <t>RED BULL VENDING MACHINE</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>15004</t>
+          <t>120001</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>1145 MCBRIDE AVE</t>
+          <t>150 WAGARAW RD</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>HAWTHORNE</t>
         </is>
       </c>
       <c r="M15" s="2" t="n"/>
-      <c r="N15" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -1649,17 +1651,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/09/2026 04:48 PM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1675,45 +1677,39 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>HILTON HASBRK HTS #50591</t>
+          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>34018</t>
+          <t>15004</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>650 TERRACE AVE</t>
+          <t>1145 MCBRIDE AVE</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>HASBROUCK HEIGHTS</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Drink Special</t>
-        </is>
-      </c>
+          <t>WOODLAND PARK</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1735,7 +1731,7 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1794,15 +1790,96 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
+          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q17" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>HILTON HASBRK HTS #50591</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>34018</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>650 TERRACE AVE</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>HASBROUCK HEIGHTS</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Drink Special</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
           <t>BARDSTOWN BOURBON COLLAB SERIES GOOSE ISLAND</t>
         </is>
       </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="P18" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COMPANY</t>
         </is>
       </c>
-      <c r="Q17" s="3" t="inlineStr">
+      <c r="Q18" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -1826,6 +1903,7 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q15" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
On-prem MPO: September refresh -- Fever Tree, Carbliss, HUSA exports + Promos_Report_36
Fever Tree 23 -> 25 new placements (Nick Melissari at goal), Carbliss
69 -> 76 new buying accounts (Nick Melissari at goal), HUSA 2 -> 3 new
draft lines (Nick Melissari at goal), Bardstown 16 -> 23 menu placements
(Allison Scott at goal). One Carbliss row (Derrick Laws / Krystal Bar)
dropped out of the new export and was not carried forward, per the
export-is-the-record rule.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N6i3Awj5JxMiknpRTkzeGy
</commit_message>
<xml_diff>
--- a/MPOs/on-prem/bardstown_menu_promos.xlsx
+++ b/MPOs/on-prem/bardstown_menu_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q18"/>
+  <dimension ref="A1:Q25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/24/2026 03:54 PM</t>
+          <t>09/28/2026 10:53 AM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -612,46 +612,44 @@
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>HUDSON FARM CLUB</t>
+          <t>BIAGIO'S</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>230126</t>
+          <t>80040</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>270 STANHOPE SPARTA RD</t>
+          <t>299 PARAMUS RD</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>ANDOVER</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N2" s="2" t="n"/>
+          <t>PARAMUS</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Menu, Weekend Promo</t>
+        </is>
+      </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -668,17 +666,17 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:11 PM</t>
+          <t>09/25/2026 08:46 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -700,33 +698,33 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -743,17 +741,17 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/25/2026 08:44 PM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -775,33 +773,33 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>BASK 46</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>15074</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>1530 RT 46 WEST</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>WOODLAND PARK</t>
         </is>
       </c>
       <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -818,17 +816,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/25/2026 08:43 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -850,33 +848,33 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>THATCHER MC GHEES (A)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>8015</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>6 WANAQUE AVE</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>POMPTON LAKES</t>
         </is>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -893,17 +891,17 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:08 PM</t>
+          <t>09/25/2026 08:36 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -925,33 +923,33 @@
       <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Weekday Promo</t>
         </is>
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -968,17 +966,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:01 PM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -989,44 +987,46 @@
       <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="n"/>
-      <c r="N7" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>PARK RIDGE</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1043,12 +1043,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1058,14 +1058,10 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Sales Associate</t>
@@ -1073,37 +1069,41 @@
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
+          <t>Promo Event Activation</t>
         </is>
       </c>
       <c r="H8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n"/>
+          <t>PARK RIDGE</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1120,12 +1120,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/24/2026 03:54 PM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1135,14 +1135,10 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
           <t>Sales Associate</t>
@@ -1150,37 +1146,41 @@
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
+          <t>Promo Event Activation</t>
         </is>
       </c>
       <c r="H9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>HUDSON FARM CLUB</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230126</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>270 STANHOPE SPARTA RD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n"/>
+          <t>ANDOVER</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
       <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1197,17 +1197,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 05:28 PM</t>
+          <t>09/16/2026 02:11 PM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1229,22 +1229,22 @@
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M10" s="2" t="n"/>
@@ -1255,7 +1255,7 @@
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1272,67 +1272,65 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n"/>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="n"/>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1349,67 +1347,65 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="n"/>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>
-      <c r="N12" s="2" t="n"/>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1426,67 +1422,65 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:08 PM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n"/>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
-      <c r="N13" s="2" t="n"/>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1503,17 +1497,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:53 AM</t>
+          <t>09/16/2026 02:01 PM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1535,33 +1529,33 @@
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK TAV (A)</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>31027</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>250 PARK AVE</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M14" s="2" t="n"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Table Tent, Menu</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1578,28 +1572,32 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:51 AM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
@@ -1612,22 +1610,22 @@
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>RED BULL VENDING MACHINE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>120001</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>150 WAGARAW RD</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M15" s="2" t="n"/>
@@ -1651,62 +1649,64 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 04:48 PM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>15004</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>1145 MCBRIDE AVE</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M16" s="2" t="n"/>
-      <c r="N16" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
           <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
@@ -1726,17 +1726,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/15/2026 05:28 PM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1752,45 +1752,39 @@
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>HILTON HASBRK HTS #50591</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>34018</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>650 TERRACE AVE</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>HASBROUCK HEIGHTS</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Drink Special</t>
-        </is>
-      </c>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n"/>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1807,33 +1801,37 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
+          <t>Feature Activation</t>
         </is>
       </c>
       <c r="H18" s="2" t="n">
@@ -1841,45 +1839,576 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="n"/>
+      <c r="N18" s="2" t="n"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q18" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>09/12/2026 08:56 AM</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Adam Badalamenti</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Sales Associate</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q19" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>09/12/2026 08:56 AM</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Adam Badalamenti</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Sales Associate</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="n"/>
+      <c r="N20" s="2" t="n"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q20" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2026 08:53 AM</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Nicholas Melissari</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n"/>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="n"/>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>NEW PARK TAV (A)</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>31027</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>250 PARK AVE</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>EAST RUTHERFORD</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="n"/>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent, Menu</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q21" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2026 08:51 AM</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Nicholas Melissari</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>RED BULL VENDING MACHINE</t>
+        </is>
+      </c>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>120001</t>
+        </is>
+      </c>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>150 WAGARAW RD</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="n"/>
+      <c r="N22" s="2" t="n"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q22" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>09/09/2026 04:48 PM</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>allison scott</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>1145 MCBRIDE AVE</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>WOODLAND PARK</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="n"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q23" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
           <t>HILTON HASBRK HTS #50591</t>
         </is>
       </c>
-      <c r="J18" s="2" t="inlineStr">
+      <c r="J24" s="2" t="inlineStr">
         <is>
           <t>34018</t>
         </is>
       </c>
-      <c r="K18" s="2" t="inlineStr">
+      <c r="K24" s="2" t="inlineStr">
         <is>
           <t>650 TERRACE AVE</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
+      <c r="L24" s="2" t="inlineStr">
         <is>
           <t>HASBROUCK HEIGHTS</t>
         </is>
       </c>
-      <c r="M18" s="2" t="inlineStr">
+      <c r="M24" s="2" t="inlineStr">
         <is>
           <t>Drink Special</t>
         </is>
       </c>
-      <c r="N18" s="2" t="inlineStr">
+      <c r="N24" s="2" t="inlineStr">
         <is>
           <t>Table Tent</t>
         </is>
       </c>
-      <c r="O18" s="2" t="inlineStr">
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q24" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>HILTON HASBRK HTS #50591</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>34018</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>650 TERRACE AVE</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>HASBROUCK HEIGHTS</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>Drink Special</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COLLAB SERIES GOOSE ISLAND</t>
         </is>
       </c>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="P25" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COMPANY</t>
         </is>
       </c>
-      <c r="Q18" s="3" t="inlineStr">
+      <c r="Q25" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -1904,6 +2433,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q16" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q17" r:id="rId16"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1960,7 +2496,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
On-prem MPOs: refresh September with 9/29 RDE exports and Promos report
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UVUQehgcyBsBQUspTHT6Gv
</commit_message>
<xml_diff>
--- a/MPOs/on-prem/bardstown_menu_promos.xlsx
+++ b/MPOs/on-prem/bardstown_menu_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q25"/>
+  <dimension ref="A1:Q32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,7 +591,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:53 AM</t>
+          <t>09/29/2026 09:56 AM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -601,7 +601,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -623,33 +623,33 @@
       <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>BIAGIO'S</t>
+          <t>ANDIAMO</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>80040</t>
+          <t>61004</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>299 PARAMUS RD</t>
+          <t>23 HARDENBURGH AVE</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>PARAMUS</t>
+          <t>HAWORTH</t>
         </is>
       </c>
       <c r="M2" s="2" t="n"/>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Menu, Weekend Promo</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -666,7 +666,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:46 PM</t>
+          <t>09/29/2026 09:54 AM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
@@ -676,7 +676,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -698,33 +698,33 @@
       <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>DUFFY'S TAVERN (Z)</t>
+          <t>BACARI</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>21043</t>
+          <t>86007</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>856 RIVER STREET</t>
+          <t>800 RIDGEWOOD RD</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WASHINGTON TWSP</t>
         </is>
       </c>
       <c r="M3" s="2" t="n"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Spirit List</t>
         </is>
       </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -741,7 +741,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:44 PM</t>
+          <t>09/29/2026 09:49 AM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -751,7 +751,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -773,33 +773,33 @@
       <c r="H4" s="2" t="n"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>BASK 46</t>
+          <t>ANDIAMO</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>15074</t>
+          <t>61004</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>1530 RT 46 WEST</t>
+          <t>23 HARDENBURGH AVE</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>HAWORTH</t>
         </is>
       </c>
       <c r="M4" s="2" t="n"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -816,12 +816,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:43 PM</t>
+          <t>09/28/2026 07:21 PM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -848,22 +848,22 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>THATCHER MC GHEES (A)</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>8015</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>6 WANAQUE AVE</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>POMPTON LAKES</t>
+          <t>HAWTHORNE</t>
         </is>
       </c>
       <c r="M5" s="2" t="n"/>
@@ -874,7 +874,7 @@
       </c>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -891,65 +891,71 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:36 PM</t>
+          <t>09/28/2026 05:03 PM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="n"/>
+          <t>Mike Kennedy</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>DUFFY'S TAVERN (Z)</t>
+          <t>MOUNTAIN RIDGE CC</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>21043</t>
+          <t>150110</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>856 RIVER STREET</t>
+          <t>713 PASSAIC AVE</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n"/>
-      <c r="N6" s="2" t="inlineStr">
-        <is>
-          <t>Weekday Promo</t>
-        </is>
-      </c>
+          <t>WEST CALDWELL</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -966,12 +972,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 04:36 PM</t>
+          <t>09/28/2026 05:03 PM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -981,10 +987,14 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="n"/>
+          <t>Mike Kennedy</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
           <t>Sales Associate</t>
@@ -1000,22 +1010,22 @@
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>PARK STEAKHOUSE</t>
+          <t>MOUNTAIN RIDGE CC</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>71005</t>
+          <t>150110</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>151 KINDERKAMACK RD</t>
+          <t>713 PASSAIC AVE</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>PARK RIDGE</t>
+          <t>WEST CALDWELL</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
@@ -1026,7 +1036,7 @@
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1043,17 +1053,17 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 04:36 PM</t>
+          <t>09/28/2026 12:57 PM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>robin feldman</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1064,46 +1074,44 @@
       <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>PARK STEAKHOUSE</t>
+          <t>THE VILLAGE INN</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>71005</t>
+          <t>12023</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>151 KINDERKAMACK RD</t>
+          <t>422 RUNNYMEDE DRIVE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>PARK RIDGE</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="n"/>
+          <t>WAYNE</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Weekend Promo</t>
+        </is>
+      </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT RYE WHISKEY</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1120,7 +1128,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/24/2026 03:54 PM</t>
+          <t>09/28/2026 10:53 AM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
@@ -1130,7 +1138,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1141,46 +1149,44 @@
       <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>HUDSON FARM CLUB</t>
+          <t>BIAGIO'S</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>230126</t>
+          <t>80040</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>270 STANHOPE SPARTA RD</t>
+          <t>299 PARAMUS RD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>ANDOVER</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="n"/>
+          <t>PARAMUS</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Menu, Weekend Promo</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1197,17 +1203,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:11 PM</t>
+          <t>09/25/2026 08:46 PM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1229,33 +1235,33 @@
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1272,17 +1278,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/25/2026 08:44 PM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1304,33 +1310,33 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>BASK 46</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>15074</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>1530 RT 46 WEST</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>WOODLAND PARK</t>
         </is>
       </c>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1347,17 +1353,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/25/2026 08:43 PM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1379,33 +1385,33 @@
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>THATCHER MC GHEES (A)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>8015</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>6 WANAQUE AVE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>POMPTON LAKES</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1422,17 +1428,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:08 PM</t>
+          <t>09/25/2026 08:36 PM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1454,33 +1460,33 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Weekday Promo</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1497,17 +1503,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:01 PM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1518,44 +1524,46 @@
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n"/>
-      <c r="N14" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>PARK RIDGE</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1572,12 +1580,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1587,14 +1595,10 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
           <t>Sales Associate</t>
@@ -1602,37 +1606,41 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
+          <t>Promo Event Activation</t>
         </is>
       </c>
       <c r="H15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n"/>
+          <t>PARK RIDGE</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -1649,12 +1657,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/24/2026 03:54 PM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1664,14 +1672,10 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
           <t>Sales Associate</t>
@@ -1679,37 +1683,41 @@
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
+          <t>Promo Event Activation</t>
         </is>
       </c>
       <c r="H16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>HUDSON FARM CLUB</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230126</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>270 STANHOPE SPARTA RD</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n"/>
+          <t>ANDOVER</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1726,17 +1734,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 05:28 PM</t>
+          <t>09/16/2026 02:11 PM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1758,22 +1766,22 @@
       <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M17" s="2" t="n"/>
@@ -1784,7 +1792,7 @@
       </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1801,67 +1809,65 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n"/>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="n"/>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -1878,67 +1884,65 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n"/>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="n"/>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1955,67 +1959,65 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 02:08 PM</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n"/>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="n"/>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2032,17 +2034,17 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:53 AM</t>
+          <t>09/16/2026 02:01 PM</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -2064,33 +2066,33 @@
       <c r="H21" s="2" t="n"/>
       <c r="I21" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK TAV (A)</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>31027</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
         <is>
-          <t>250 PARK AVE</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M21" s="2" t="n"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Table Tent, Menu</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2107,28 +2109,32 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:51 AM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2141,22 +2147,22 @@
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>RED BULL VENDING MACHINE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>120001</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>150 WAGARAW RD</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M22" s="2" t="n"/>
@@ -2180,62 +2186,64 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 04:48 PM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>15004</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>1145 MCBRIDE AVE</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="inlineStr">
         <is>
           <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
@@ -2255,17 +2263,17 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/15/2026 05:28 PM</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2281,45 +2289,39 @@
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>HILTON HASBRK HTS #50591</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>34018</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>650 TERRACE AVE</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>HASBROUCK HEIGHTS</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>Drink Special</t>
-        </is>
-      </c>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="n"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Menu</t>
         </is>
       </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2336,33 +2338,37 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
+          <t>Feature Activation</t>
         </is>
       </c>
       <c r="H25" s="2" t="n">
@@ -2370,45 +2376,576 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="n"/>
+      <c r="N25" s="2" t="n"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q25" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>09/12/2026 08:56 AM</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Adam Badalamenti</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Sales Associate</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="n"/>
+      <c r="N26" s="2" t="n"/>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q26" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>09/12/2026 08:56 AM</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Adam Badalamenti</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Sales Associate</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>191710</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>90 ROUTE 206</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="inlineStr">
+        <is>
+          <t>STANHOPE</t>
+        </is>
+      </c>
+      <c r="M27" s="2" t="n"/>
+      <c r="N27" s="2" t="n"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P27" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q27" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2026 08:53 AM</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Nicholas Melissari</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>NEW PARK TAV (A)</t>
+        </is>
+      </c>
+      <c r="J28" s="2" t="inlineStr">
+        <is>
+          <t>31027</t>
+        </is>
+      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>250 PARK AVE</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>EAST RUTHERFORD</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent, Menu</t>
+        </is>
+      </c>
+      <c r="O28" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q28" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>09/11/2026 08:51 AM</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Nicholas Melissari</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n"/>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>RED BULL VENDING MACHINE</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>120001</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>150 WAGARAW RD</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="inlineStr">
+        <is>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M29" s="2" t="n"/>
+      <c r="N29" s="2" t="n"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+        </is>
+      </c>
+      <c r="P29" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q29" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>09/09/2026 04:48 PM</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>2.1</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>allison scott</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="n"/>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+        </is>
+      </c>
+      <c r="J30" s="2" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="K30" s="2" t="inlineStr">
+        <is>
+          <t>1145 MCBRIDE AVE</t>
+        </is>
+      </c>
+      <c r="L30" s="2" t="inlineStr">
+        <is>
+          <t>WOODLAND PARK</t>
+        </is>
+      </c>
+      <c r="M30" s="2" t="n"/>
+      <c r="N30" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+        </is>
+      </c>
+      <c r="P30" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q30" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
           <t>HILTON HASBRK HTS #50591</t>
         </is>
       </c>
-      <c r="J25" s="2" t="inlineStr">
+      <c r="J31" s="2" t="inlineStr">
         <is>
           <t>34018</t>
         </is>
       </c>
-      <c r="K25" s="2" t="inlineStr">
+      <c r="K31" s="2" t="inlineStr">
         <is>
           <t>650 TERRACE AVE</t>
         </is>
       </c>
-      <c r="L25" s="2" t="inlineStr">
+      <c r="L31" s="2" t="inlineStr">
         <is>
           <t>HASBROUCK HEIGHTS</t>
         </is>
       </c>
-      <c r="M25" s="2" t="inlineStr">
+      <c r="M31" s="2" t="inlineStr">
         <is>
           <t>Drink Special</t>
         </is>
       </c>
-      <c r="N25" s="2" t="inlineStr">
+      <c r="N31" s="2" t="inlineStr">
         <is>
           <t>Table Tent</t>
         </is>
       </c>
-      <c r="O25" s="2" t="inlineStr">
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+        </is>
+      </c>
+      <c r="P31" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q31" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E32" s="2" t="n"/>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>HILTON HASBRK HTS #50591</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>34018</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>650 TERRACE AVE</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>HASBROUCK HEIGHTS</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="inlineStr">
+        <is>
+          <t>Drink Special</t>
+        </is>
+      </c>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COLLAB SERIES GOOSE ISLAND</t>
         </is>
       </c>
-      <c r="P25" s="2" t="inlineStr">
+      <c r="P32" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COMPANY</t>
         </is>
       </c>
-      <c r="Q25" s="3" t="inlineStr">
+      <c r="Q32" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -2440,6 +2977,13 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q23" r:id="rId22"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q24" r:id="rId23"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId31"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
On-prem MPOs: 9/30 refresh -- Promos_Report_38 merged, exports unchanged
The Fever Tree, Carbliss and HUSA exports match the 9/29 pull row for
row. Report_38 adds two Bardstown rows at an off-premise account
(skipped by the on-premise-only rule), so every rep's September number
holds; sync_meta re-stamped.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01MKEPYk6YSQsdW7mR8WAxwM
</commit_message>
<xml_diff>
--- a/MPOs/on-prem/bardstown_menu_promos.xlsx
+++ b/MPOs/on-prem/bardstown_menu_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q32"/>
+  <dimension ref="A1:Q34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,25 +591,29 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 09:56 AM</t>
+          <t>09/30/2026 09:57 AM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Paul McLaughlin</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="n"/>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
@@ -617,39 +621,37 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>ANDIAMO</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>61004</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>23 HARDENBURGH AVE</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>HAWORTH</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N2" s="2" t="n"/>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT BOURBON WHISKEY</t>
+          <t>GREEN RIVER ARMY 250TH ANNIVERSARY</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -666,25 +668,29 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 09:54 AM</t>
+          <t>09/30/2026 09:57 AM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Paul McLaughlin</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="n"/>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
@@ -692,39 +698,37 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>BACARI</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>86007</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>800 RIDGEWOOD RD</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>WASHINGTON TWSP</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="inlineStr">
-        <is>
-          <t>Spirit List</t>
-        </is>
-      </c>
+      <c r="N3" s="2" t="n"/>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -741,12 +745,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 09:49 AM</t>
+          <t>09/29/2026 09:56 AM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -799,7 +803,7 @@
       </c>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -816,17 +820,17 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 07:21 PM</t>
+          <t>09/29/2026 09:54 AM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -848,28 +852,28 @@
       <c r="H5" s="2" t="n"/>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>BACARI</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>86007</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>800 RIDGEWOOD RD</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>WASHINGTON TWSP</t>
         </is>
       </c>
       <c r="M5" s="2" t="n"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Spirit List</t>
         </is>
       </c>
       <c r="O5" s="2" t="inlineStr">
@@ -891,71 +895,65 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 05:03 PM</t>
+          <t>09/29/2026 09:49 AM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Mike Kennedy</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="n"/>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="n"/>
       <c r="I6" s="2" t="inlineStr">
         <is>
-          <t>MOUNTAIN RIDGE CC</t>
+          <t>ANDIAMO</t>
         </is>
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>150110</t>
+          <t>61004</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>713 PASSAIC AVE</t>
+          <t>23 HARDENBURGH AVE</t>
         </is>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>WEST CALDWELL</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N6" s="2" t="n"/>
+          <t>HAWORTH</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="n"/>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -972,71 +970,65 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 05:03 PM</t>
+          <t>09/28/2026 07:21 PM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Mike Kennedy</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n"/>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>MOUNTAIN RIDGE CC</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>150110</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>713 PASSAIC AVE</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>WEST CALDWELL</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N7" s="2" t="n"/>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="n"/>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
       <c r="O7" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P7" s="2" t="inlineStr">
@@ -1053,65 +1045,71 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 12:57 PM</t>
+          <t>09/28/2026 05:03 PM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="n"/>
+          <t>Mike Kennedy</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>THE VILLAGE INN</t>
+          <t>MOUNTAIN RIDGE CC</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>12023</t>
+          <t>150110</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>422 RUNNYMEDE DRIVE</t>
+          <t>713 PASSAIC AVE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>WAYNE</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n"/>
-      <c r="N8" s="2" t="inlineStr">
-        <is>
-          <t>Weekend Promo</t>
-        </is>
-      </c>
+          <t>WEST CALDWELL</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT RYE WHISKEY</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1128,65 +1126,71 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:53 AM</t>
+          <t>09/28/2026 05:03 PM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="n"/>
+          <t>Mike Kennedy</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>BIAGIO'S</t>
+          <t>MOUNTAIN RIDGE CC</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>80040</t>
+          <t>150110</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>299 PARAMUS RD</t>
+          <t>713 PASSAIC AVE</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>PARAMUS</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n"/>
-      <c r="N9" s="2" t="inlineStr">
-        <is>
-          <t>Menu, Weekend Promo</t>
-        </is>
-      </c>
+          <t>WEST CALDWELL</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="n"/>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1203,17 +1207,17 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:46 PM</t>
+          <t>09/28/2026 12:57 PM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>robin feldman</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1235,33 +1239,33 @@
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>DUFFY'S TAVERN (Z)</t>
+          <t>THE VILLAGE INN</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>21043</t>
+          <t>12023</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>856 RIVER STREET</t>
+          <t>422 RUNNYMEDE DRIVE</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WAYNE</t>
         </is>
       </c>
       <c r="M10" s="2" t="n"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Weekend Promo</t>
         </is>
       </c>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT RYE WHISKEY</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1278,17 +1282,17 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:44 PM</t>
+          <t>09/28/2026 10:53 AM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1310,33 +1314,33 @@
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>BASK 46</t>
+          <t>BIAGIO'S</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>15074</t>
+          <t>80040</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>1530 RT 46 WEST</t>
+          <t>299 PARAMUS RD</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>PARAMUS</t>
         </is>
       </c>
       <c r="M11" s="2" t="n"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Menu, Weekend Promo</t>
         </is>
       </c>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1353,12 +1357,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:43 PM</t>
+          <t>09/25/2026 08:46 PM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1385,22 +1389,22 @@
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>THATCHER MC GHEES (A)</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>8015</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>6 WANAQUE AVE</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>POMPTON LAKES</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>
@@ -1428,12 +1432,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:36 PM</t>
+          <t>09/25/2026 08:44 PM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1460,28 +1464,28 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>DUFFY'S TAVERN (Z)</t>
+          <t>BASK 46</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>21043</t>
+          <t>15074</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>856 RIVER STREET</t>
+          <t>1530 RT 46 WEST</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WOODLAND PARK</t>
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Weekday Promo</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
@@ -1503,17 +1507,17 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 04:36 PM</t>
+          <t>09/25/2026 08:43 PM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1524,46 +1528,44 @@
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>PARK STEAKHOUSE</t>
+          <t>THATCHER MC GHEES (A)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>71005</t>
+          <t>8015</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>151 KINDERKAMACK RD</t>
+          <t>6 WANAQUE AVE</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>PARK RIDGE</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N14" s="2" t="n"/>
+          <t>POMPTON LAKES</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="n"/>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
       <c r="O14" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P14" s="2" t="inlineStr">
@@ -1580,17 +1582,17 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 04:36 PM</t>
+          <t>09/25/2026 08:36 PM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1601,46 +1603,44 @@
       <c r="E15" s="2" t="n"/>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>PARK STEAKHOUSE</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>71005</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>151 KINDERKAMACK RD</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>PARK RIDGE</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N15" s="2" t="n"/>
+          <t>PATERSON</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="n"/>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>Weekday Promo</t>
+        </is>
+      </c>
       <c r="O15" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P15" s="2" t="inlineStr">
@@ -1657,12 +1657,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/24/2026 03:54 PM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1691,22 +1691,22 @@
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>HUDSON FARM CLUB</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>230126</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>270 STANHOPE SPARTA RD</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>ANDOVER</t>
+          <t>PARK RIDGE</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
@@ -1734,17 +1734,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:11 PM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1755,44 +1755,46 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n"/>
-      <c r="N17" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>PARK RIDGE</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1809,17 +1811,17 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/24/2026 03:54 PM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1830,44 +1832,46 @@
       <c r="E18" s="2" t="n"/>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>HUDSON FARM CLUB</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>230126</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>270 STANHOPE SPARTA RD</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n"/>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>ANDOVER</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P18" s="2" t="inlineStr">
@@ -1884,12 +1888,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/16/2026 02:11 PM</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1942,7 +1946,7 @@
       </c>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1959,12 +1963,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:08 PM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -2017,7 +2021,7 @@
       </c>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2034,12 +2038,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:01 PM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2092,7 +2096,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2109,55 +2113,49 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:08 PM</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E22" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="n"/>
       <c r="I22" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L22" s="2" t="inlineStr">
@@ -2166,10 +2164,14 @@
         </is>
       </c>
       <c r="M22" s="2" t="n"/>
-      <c r="N22" s="2" t="n"/>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2186,55 +2188,49 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:01 PM</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E23" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H23" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="n"/>
       <c r="I23" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L23" s="2" t="inlineStr">
@@ -2243,10 +2239,14 @@
         </is>
       </c>
       <c r="M23" s="2" t="n"/>
-      <c r="N23" s="2" t="n"/>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2263,65 +2263,67 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 05:28 PM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N24" s="2" t="n"/>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2338,12 +2340,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2376,29 +2378,29 @@
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M25" s="2" t="n"/>
       <c r="N25" s="2" t="n"/>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -2415,67 +2417,65 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/15/2026 05:28 PM</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="n"/>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n"/>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>HAWTHORNE</t>
         </is>
       </c>
       <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="n"/>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -2497,7 +2497,7 @@
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2552,7 +2552,7 @@
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -2569,65 +2569,67 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:53 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK TAV (A)</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>31027</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>250 PARK AVE</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>STANHOPE</t>
         </is>
       </c>
       <c r="M28" s="2" t="n"/>
-      <c r="N28" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent, Menu</t>
-        </is>
-      </c>
+      <c r="N28" s="2" t="n"/>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -2644,28 +2646,32 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:51 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E29" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
@@ -2678,22 +2684,22 @@
       </c>
       <c r="I29" s="2" t="inlineStr">
         <is>
-          <t>RED BULL VENDING MACHINE</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J29" s="2" t="inlineStr">
         <is>
-          <t>120001</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>150 WAGARAW RD</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L29" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>STANHOPE</t>
         </is>
       </c>
       <c r="M29" s="2" t="n"/>
@@ -2717,17 +2723,17 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 04:48 PM</t>
+          <t>09/11/2026 08:53 AM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2749,33 +2755,33 @@
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+          <t>NEW PARK TAV (A)</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>15004</t>
+          <t>31027</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>1145 MCBRIDE AVE</t>
+          <t>250 PARK AVE</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>EAST RUTHERFORD</t>
         </is>
       </c>
       <c r="M30" s="2" t="n"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent, Menu</t>
         </is>
       </c>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -2792,17 +2798,17 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/11/2026 08:51 AM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2818,7 +2824,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
+          <t>Feature Activation</t>
         </is>
       </c>
       <c r="H31" s="2" t="n">
@@ -2826,37 +2832,29 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>HILTON HASBRK HTS #50591</t>
+          <t>RED BULL VENDING MACHINE</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>34018</t>
+          <t>120001</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>650 TERRACE AVE</t>
+          <t>150 WAGARAW RD</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>HASBROUCK HEIGHTS</t>
-        </is>
-      </c>
-      <c r="M31" s="2" t="inlineStr">
-        <is>
-          <t>Drink Special</t>
-        </is>
-      </c>
-      <c r="N31" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent</t>
-        </is>
-      </c>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="n"/>
+      <c r="N31" s="2" t="n"/>
       <c r="O31" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P31" s="2" t="inlineStr">
@@ -2873,17 +2871,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/09/2026 04:48 PM</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2899,53 +2897,209 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="n"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+        </is>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="K32" s="2" t="inlineStr">
+        <is>
+          <t>1145 MCBRIDE AVE</t>
+        </is>
+      </c>
+      <c r="L32" s="2" t="inlineStr">
+        <is>
+          <t>WOODLAND PARK</t>
+        </is>
+      </c>
+      <c r="M32" s="2" t="n"/>
+      <c r="N32" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+        </is>
+      </c>
+      <c r="P32" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q32" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n"/>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
           <t>Feature Activation (on)</t>
         </is>
       </c>
-      <c r="H32" s="2" t="n">
+      <c r="H33" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I33" s="2" t="inlineStr">
         <is>
           <t>HILTON HASBRK HTS #50591</t>
         </is>
       </c>
-      <c r="J32" s="2" t="inlineStr">
+      <c r="J33" s="2" t="inlineStr">
         <is>
           <t>34018</t>
         </is>
       </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="K33" s="2" t="inlineStr">
         <is>
           <t>650 TERRACE AVE</t>
         </is>
       </c>
-      <c r="L32" s="2" t="inlineStr">
+      <c r="L33" s="2" t="inlineStr">
         <is>
           <t>HASBROUCK HEIGHTS</t>
         </is>
       </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="M33" s="2" t="inlineStr">
         <is>
           <t>Drink Special</t>
         </is>
       </c>
-      <c r="N32" s="2" t="inlineStr">
+      <c r="N33" s="2" t="inlineStr">
         <is>
           <t>Table Tent</t>
         </is>
       </c>
-      <c r="O32" s="2" t="inlineStr">
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+        </is>
+      </c>
+      <c r="P33" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q33" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D34" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E34" s="2" t="n"/>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>HILTON HASBRK HTS #50591</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>34018</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>650 TERRACE AVE</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>HASBROUCK HEIGHTS</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="inlineStr">
+        <is>
+          <t>Drink Special</t>
+        </is>
+      </c>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COLLAB SERIES GOOSE ISLAND</t>
         </is>
       </c>
-      <c r="P32" s="2" t="inlineStr">
+      <c r="P34" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COMPANY</t>
         </is>
       </c>
-      <c r="Q32" s="3" t="inlineStr">
+      <c r="Q34" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -2984,6 +3138,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q30" r:id="rId29"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q31" r:id="rId30"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId33"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
On-prem MPOs: 10/1 refresh -- Carbliss export, Promos_Report_42 merged
Final September pull. Fever Tree and HUSA exports identical to the 9/30
files (27 / 3 hold). Carbliss 101 -> 100: Anthony Palmisano's 9/30 Doc's
Place row left the export (7 -> 6). Bardstown 30 -> 32 menu placements:
Allison Scott's two 9/30 Green River Honey cocktail lists (7 -> 9).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FtE2WbdaY1rMKAtZ5xxusS
</commit_message>
<xml_diff>
--- a/MPOs/on-prem/bardstown_menu_promos.xlsx
+++ b/MPOs/on-prem/bardstown_menu_promos.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q34"/>
+  <dimension ref="A1:Q36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21.7109375" customWidth="1" style="6" min="1" max="1"/>
@@ -591,29 +591,25 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>09/30/2026 09:57 AM</t>
+          <t>09/30/2026 08:26 PM</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
@@ -621,37 +617,39 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>2</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="n"/>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>THE LITTLE FALLS TAVERN</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>13002</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>131 NEWARK POMPTON TURNPIKE</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>LITTLE FALLS</t>
         </is>
       </c>
       <c r="M2" s="2" t="n"/>
-      <c r="N2" s="2" t="n"/>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O2" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER ARMY 250TH ANNIVERSARY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P2" s="2" t="inlineStr">
@@ -668,29 +666,25 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>09/30/2026 09:57 AM</t>
+          <t>09/30/2026 08:23 PM</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>2.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Chris Payton</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Michael Engel</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
@@ -698,37 +692,39 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="n">
-        <v>3</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="n"/>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
+          <t>WAYNE ALE HOUSE &amp; PIZZA</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>76010</t>
+          <t>12026</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>66 MARKET ST</t>
+          <t>611 RATZER ROAD</t>
         </is>
       </c>
       <c r="L3" s="2" t="inlineStr">
         <is>
-          <t>SADDLE BROOK</t>
+          <t>WAYNE</t>
         </is>
       </c>
       <c r="M3" s="2" t="n"/>
-      <c r="N3" s="2" t="n"/>
+      <c r="N3" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O3" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P3" s="2" t="inlineStr">
@@ -745,25 +741,29 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 09:56 AM</t>
+          <t>09/30/2026 09:57 AM</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Paul McLaughlin</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="n"/>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
@@ -771,39 +771,37 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>2</v>
+      </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>ANDIAMO</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>61004</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>23 HARDENBURGH AVE</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>HAWORTH</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M4" s="2" t="n"/>
-      <c r="N4" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT BOURBON WHISKEY</t>
+          <t>GREEN RIVER ARMY 250TH ANNIVERSARY</t>
         </is>
       </c>
       <c r="P4" s="2" t="inlineStr">
@@ -820,25 +818,29 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 09:54 AM</t>
+          <t>09/30/2026 09:57 AM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>2.2</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Paul McLaughlin</t>
+          <t>Chris Payton</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="n"/>
+          <t>Michael Engel</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
           <t>Sales Rep</t>
@@ -846,39 +848,37 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>3</v>
+      </c>
       <c r="I5" s="2" t="inlineStr">
         <is>
-          <t>BACARI</t>
+          <t>USA WINE TRADERS CLUB (SADDLE BROOK)</t>
         </is>
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>86007</t>
+          <t>76010</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
         <is>
-          <t>800 RIDGEWOOD RD</t>
+          <t>66 MARKET ST</t>
         </is>
       </c>
       <c r="L5" s="2" t="inlineStr">
         <is>
-          <t>WASHINGTON TWSP</t>
+          <t>SADDLE BROOK</t>
         </is>
       </c>
       <c r="M5" s="2" t="n"/>
-      <c r="N5" s="2" t="inlineStr">
-        <is>
-          <t>Spirit List</t>
-        </is>
-      </c>
+      <c r="N5" s="2" t="n"/>
       <c r="O5" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P5" s="2" t="inlineStr">
@@ -895,12 +895,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>09/29/2026 09:49 AM</t>
+          <t>09/29/2026 09:56 AM</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -953,7 +953,7 @@
       </c>
       <c r="O6" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P6" s="2" t="inlineStr">
@@ -970,17 +970,17 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 07:21 PM</t>
+          <t>09/29/2026 09:54 AM</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -1002,28 +1002,28 @@
       <c r="H7" s="2" t="n"/>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>BACARI</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>86007</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>800 RIDGEWOOD RD</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>WASHINGTON TWSP</t>
         </is>
       </c>
       <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Spirit List</t>
         </is>
       </c>
       <c r="O7" s="2" t="inlineStr">
@@ -1045,71 +1045,65 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 05:03 PM</t>
+          <t>09/29/2026 09:49 AM</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>Paul McLaughlin</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Mike Kennedy</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="n"/>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="n"/>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>MOUNTAIN RIDGE CC</t>
+          <t>ANDIAMO</t>
         </is>
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>150110</t>
+          <t>61004</t>
         </is>
       </c>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>713 PASSAIC AVE</t>
+          <t>23 HARDENBURGH AVE</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>WEST CALDWELL</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N8" s="2" t="n"/>
+          <t>HAWORTH</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="n"/>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O8" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P8" s="2" t="inlineStr">
@@ -1126,71 +1120,65 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 05:03 PM</t>
+          <t>09/28/2026 07:21 PM</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Mike Kennedy</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n"/>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>MOUNTAIN RIDGE CC</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>150110</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>713 PASSAIC AVE</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>WEST CALDWELL</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N9" s="2" t="n"/>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="n"/>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
       <c r="O9" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P9" s="2" t="inlineStr">
@@ -1207,65 +1195,71 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 12:57 PM</t>
+          <t>09/28/2026 05:03 PM</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>7.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="n"/>
+          <t>Mike Kennedy</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>THE VILLAGE INN</t>
+          <t>MOUNTAIN RIDGE CC</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>12023</t>
+          <t>150110</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>422 RUNNYMEDE DRIVE</t>
+          <t>713 PASSAIC AVE</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>WAYNE</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n"/>
-      <c r="N10" s="2" t="inlineStr">
-        <is>
-          <t>Weekend Promo</t>
-        </is>
-      </c>
+          <t>WEST CALDWELL</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT RYE WHISKEY</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P10" s="2" t="inlineStr">
@@ -1282,65 +1276,71 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>09/28/2026 10:53 AM</t>
+          <t>09/28/2026 05:03 PM</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="n"/>
+          <t>Mike Kennedy</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>BIAGIO'S</t>
+          <t>MOUNTAIN RIDGE CC</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>80040</t>
+          <t>150110</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>299 PARAMUS RD</t>
+          <t>713 PASSAIC AVE</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>PARAMUS</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n"/>
-      <c r="N11" s="2" t="inlineStr">
-        <is>
-          <t>Menu, Weekend Promo</t>
-        </is>
-      </c>
+          <t>WEST CALDWELL</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P11" s="2" t="inlineStr">
@@ -1357,17 +1357,17 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:46 PM</t>
+          <t>09/28/2026 12:57 PM</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>7.1</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>robin feldman</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1389,33 +1389,33 @@
       <c r="H12" s="2" t="n"/>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>DUFFY'S TAVERN (Z)</t>
+          <t>THE VILLAGE INN</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>21043</t>
+          <t>12023</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>856 RIVER STREET</t>
+          <t>422 RUNNYMEDE DRIVE</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WAYNE</t>
         </is>
       </c>
       <c r="M12" s="2" t="n"/>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Weekend Promo</t>
         </is>
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT RYE WHISKEY</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
@@ -1432,17 +1432,17 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:44 PM</t>
+          <t>09/28/2026 10:53 AM</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1464,33 +1464,33 @@
       <c r="H13" s="2" t="n"/>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>BASK 46</t>
+          <t>BIAGIO'S</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>15074</t>
+          <t>80040</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>1530 RT 46 WEST</t>
+          <t>299 PARAMUS RD</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>PARAMUS</t>
         </is>
       </c>
       <c r="M13" s="2" t="n"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Table Tent</t>
+          <t>Menu, Weekend Promo</t>
         </is>
       </c>
       <c r="O13" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P13" s="2" t="inlineStr">
@@ -1507,12 +1507,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:43 PM</t>
+          <t>09/25/2026 08:46 PM</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1539,22 +1539,22 @@
       <c r="H14" s="2" t="n"/>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>THATCHER MC GHEES (A)</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>8015</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>6 WANAQUE AVE</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>POMPTON LAKES</t>
+          <t>PATERSON</t>
         </is>
       </c>
       <c r="M14" s="2" t="n"/>
@@ -1582,12 +1582,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 08:36 PM</t>
+          <t>09/25/2026 08:44 PM</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1614,28 +1614,28 @@
       <c r="H15" s="2" t="n"/>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>DUFFY'S TAVERN (Z)</t>
+          <t>BASK 46</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>21043</t>
+          <t>15074</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>856 RIVER STREET</t>
+          <t>1530 RT 46 WEST</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>PATERSON</t>
+          <t>WOODLAND PARK</t>
         </is>
       </c>
       <c r="M15" s="2" t="n"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Weekday Promo</t>
+          <t>Table Tent</t>
         </is>
       </c>
       <c r="O15" s="2" t="inlineStr">
@@ -1657,17 +1657,17 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 04:36 PM</t>
+          <t>09/25/2026 08:43 PM</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1678,46 +1678,44 @@
       <c r="E16" s="2" t="n"/>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="n"/>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>PARK STEAKHOUSE</t>
+          <t>THATCHER MC GHEES (A)</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>71005</t>
+          <t>8015</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>151 KINDERKAMACK RD</t>
+          <t>6 WANAQUE AVE</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>PARK RIDGE</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N16" s="2" t="n"/>
+          <t>POMPTON LAKES</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="n"/>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
       <c r="O16" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P16" s="2" t="inlineStr">
@@ -1734,17 +1732,17 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>09/25/2026 04:36 PM</t>
+          <t>09/25/2026 08:36 PM</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1755,46 +1753,44 @@
       <c r="E17" s="2" t="n"/>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Promo Event Activation</t>
-        </is>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>0</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="n"/>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>PARK STEAKHOUSE</t>
+          <t>DUFFY'S TAVERN (Z)</t>
         </is>
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>71005</t>
+          <t>21043</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
         <is>
-          <t>151 KINDERKAMACK RD</t>
+          <t>856 RIVER STREET</t>
         </is>
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>PARK RIDGE</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="inlineStr">
-        <is>
-          <t>Promo Tasting</t>
-        </is>
-      </c>
-      <c r="N17" s="2" t="n"/>
+          <t>PATERSON</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="n"/>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>Weekday Promo</t>
+        </is>
+      </c>
       <c r="O17" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P17" s="2" t="inlineStr">
@@ -1811,12 +1807,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>09/24/2026 03:54 PM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.1</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1845,22 +1841,22 @@
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>HUDSON FARM CLUB</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>230126</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
         <is>
-          <t>270 STANHOPE SPARTA RD</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L18" s="2" t="inlineStr">
         <is>
-          <t>ANDOVER</t>
+          <t>PARK RIDGE</t>
         </is>
       </c>
       <c r="M18" s="2" t="inlineStr">
@@ -1888,17 +1884,17 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:11 PM</t>
+          <t>09/25/2026 04:36 PM</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>6.2</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1909,44 +1905,46 @@
       <c r="E19" s="2" t="n"/>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H19" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>PARK STEAKHOUSE</t>
         </is>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>71005</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>151 KINDERKAMACK RD</t>
         </is>
       </c>
       <c r="L19" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M19" s="2" t="n"/>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>PARK RIDGE</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P19" s="2" t="inlineStr">
@@ -1963,17 +1961,17 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/24/2026 03:54 PM</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>brian sengebush</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1984,44 +1982,46 @@
       <c r="E20" s="2" t="n"/>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="n"/>
+          <t>Promo Event Activation</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="n">
+        <v>0</v>
+      </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
-          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
+          <t>HUDSON FARM CLUB</t>
         </is>
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>230122</t>
+          <t>230126</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>23 WHITE DEER PLAZA</t>
+          <t>270 STANHOPE SPARTA RD</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr">
         <is>
-          <t>SPARTA</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="n"/>
-      <c r="N20" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+          <t>ANDOVER</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>Promo Tasting</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="n"/>
       <c r="O20" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
+          <t>BARDSTOWN ORIGINS SINGLE BARREL</t>
         </is>
       </c>
       <c r="P20" s="2" t="inlineStr">
@@ -2038,12 +2038,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:10 PM</t>
+          <t>09/16/2026 02:11 PM</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -2096,7 +2096,7 @@
       </c>
       <c r="O21" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P21" s="2" t="inlineStr">
@@ -2113,12 +2113,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:08 PM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>4.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2171,7 +2171,7 @@
       </c>
       <c r="O22" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOTTLED IN BOND BOURBON</t>
         </is>
       </c>
       <c r="P22" s="2" t="inlineStr">
@@ -2188,12 +2188,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 02:01 PM</t>
+          <t>09/16/2026 02:10 PM</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>5.1</t>
+          <t>3.1</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2246,7 +2246,7 @@
       </c>
       <c r="O23" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P23" s="2" t="inlineStr">
@@ -2263,55 +2263,49 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:08 PM</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>4.1</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E24" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="n"/>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="n"/>
       <c r="I24" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L24" s="2" t="inlineStr">
@@ -2320,10 +2314,14 @@
         </is>
       </c>
       <c r="M24" s="2" t="n"/>
-      <c r="N24" s="2" t="n"/>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O24" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN WHEATED BOURBON</t>
         </is>
       </c>
       <c r="P24" s="2" t="inlineStr">
@@ -2340,55 +2338,49 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>09/16/2026 10:00 AM</t>
+          <t>09/16/2026 02:01 PM</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>5.1</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>brian sengebush</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E25" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n"/>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H25" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="n"/>
       <c r="I25" s="2" t="inlineStr">
         <is>
-          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
+          <t>KROGH'S RESTAURANT &amp; BREW PUB</t>
         </is>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>230105</t>
+          <t>230122</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>16 NORTH VILLAGE BLVD</t>
+          <t>23 WHITE DEER PLAZA</t>
         </is>
       </c>
       <c r="L25" s="2" t="inlineStr">
@@ -2397,10 +2389,14 @@
         </is>
       </c>
       <c r="M25" s="2" t="n"/>
-      <c r="N25" s="2" t="n"/>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O25" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN RYE</t>
         </is>
       </c>
       <c r="P25" s="2" t="inlineStr">
@@ -2417,65 +2413,67 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>09/15/2026 05:28 PM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E26" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I26" s="2" t="inlineStr">
         <is>
-          <t>BOTTAGRA REST (P)</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>19012</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
         <is>
-          <t>80 WAGARAW ROAD</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M26" s="2" t="n"/>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>Menu</t>
-        </is>
-      </c>
+      <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P26" s="2" t="inlineStr">
@@ -2492,12 +2490,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/16/2026 10:00 AM</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2530,29 +2528,29 @@
       </c>
       <c r="I27" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>SHOPRITE WINES &amp; SPIRITS OF SPARTA</t>
         </is>
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>230105</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>16 NORTH VILLAGE BLVD</t>
         </is>
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>SPARTA</t>
         </is>
       </c>
       <c r="M27" s="2" t="n"/>
       <c r="N27" s="2" t="n"/>
       <c r="O27" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
         </is>
       </c>
       <c r="P27" s="2" t="inlineStr">
@@ -2569,67 +2567,65 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>09/12/2026 08:56 AM</t>
+          <t>09/15/2026 05:28 PM</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Adam Badalamenti</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>Paul Deady</t>
-        </is>
-      </c>
-      <c r="E28" s="2" t="inlineStr">
-        <is>
-          <t>Ashley Furman</t>
-        </is>
-      </c>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E28" s="2" t="n"/>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>Sales Associate</t>
+          <t>Sales Rep</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="n">
-        <v>1</v>
-      </c>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="inlineStr">
         <is>
-          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
+          <t>BOTTAGRA REST (P)</t>
         </is>
       </c>
       <c r="J28" s="2" t="inlineStr">
         <is>
-          <t>191710</t>
+          <t>19012</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
         <is>
-          <t>90 ROUTE 206</t>
+          <t>80 WAGARAW ROAD</t>
         </is>
       </c>
       <c r="L28" s="2" t="inlineStr">
         <is>
-          <t>STANHOPE</t>
+          <t>HAWTHORNE</t>
         </is>
       </c>
       <c r="M28" s="2" t="n"/>
-      <c r="N28" s="2" t="n"/>
+      <c r="N28" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
       <c r="O28" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
+          <t>BARDSTOWN BOURBON CO. ORIGIN BOURBON</t>
         </is>
       </c>
       <c r="P28" s="2" t="inlineStr">
@@ -2651,7 +2647,7 @@
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>1.3</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2706,7 +2702,7 @@
       <c r="N29" s="2" t="n"/>
       <c r="O29" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN BOURBON 2026 DISCOVERY</t>
         </is>
       </c>
       <c r="P29" s="2" t="inlineStr">
@@ -2723,65 +2719,67 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:53 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1.2</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E30" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E30" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>Cocktail List Activation</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="n"/>
+          <t>Feature Activation</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="I30" s="2" t="inlineStr">
         <is>
-          <t>NEW PARK TAV (A)</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J30" s="2" t="inlineStr">
         <is>
-          <t>31027</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>250 PARK AVE</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L30" s="2" t="inlineStr">
         <is>
-          <t>EAST RUTHERFORD</t>
+          <t>STANHOPE</t>
         </is>
       </c>
       <c r="M30" s="2" t="n"/>
-      <c r="N30" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent, Menu</t>
-        </is>
-      </c>
+      <c r="N30" s="2" t="n"/>
       <c r="O30" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
+          <t>BARDSTOWN COLLABORATION SERIES LOCHS OF JURA</t>
         </is>
       </c>
       <c r="P30" s="2" t="inlineStr">
@@ -2798,28 +2796,32 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>09/11/2026 08:51 AM</t>
+          <t>09/12/2026 08:56 AM</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.3</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Nicholas Melissari</t>
+          <t>Adam Badalamenti</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Christopher McCrohan</t>
-        </is>
-      </c>
-      <c r="E31" s="2" t="n"/>
+          <t>Paul Deady</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Ashley Furman</t>
+        </is>
+      </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>Sales Rep</t>
+          <t>Sales Associate</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
@@ -2832,22 +2834,22 @@
       </c>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>RED BULL VENDING MACHINE</t>
+          <t>SHOP RITE WINE &amp; SPIRITS STANHOPE</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr">
         <is>
-          <t>120001</t>
+          <t>191710</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>150 WAGARAW RD</t>
+          <t>90 ROUTE 206</t>
         </is>
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>HAWTHORNE</t>
+          <t>STANHOPE</t>
         </is>
       </c>
       <c r="M31" s="2" t="n"/>
@@ -2871,17 +2873,17 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>09/09/2026 04:48 PM</t>
+          <t>09/11/2026 08:53 AM</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>2.1</t>
+          <t>1.1</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>allison scott</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2903,33 +2905,33 @@
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+          <t>NEW PARK TAV (A)</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
         <is>
-          <t>15004</t>
+          <t>31027</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
         <is>
-          <t>1145 MCBRIDE AVE</t>
+          <t>250 PARK AVE</t>
         </is>
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>WOODLAND PARK</t>
+          <t>EAST RUTHERFORD</t>
         </is>
       </c>
       <c r="M32" s="2" t="n"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Menu</t>
+          <t>Table Tent, Menu</t>
         </is>
       </c>
       <c r="O32" s="2" t="inlineStr">
         <is>
-          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P32" s="2" t="inlineStr">
@@ -2946,17 +2948,17 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/11/2026 08:51 AM</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>Nicholas Melissari</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2972,7 +2974,7 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Feature Activation (on)</t>
+          <t>Feature Activation</t>
         </is>
       </c>
       <c r="H33" s="2" t="n">
@@ -2980,37 +2982,29 @@
       </c>
       <c r="I33" s="2" t="inlineStr">
         <is>
-          <t>HILTON HASBRK HTS #50591</t>
+          <t>RED BULL VENDING MACHINE</t>
         </is>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
-          <t>34018</t>
+          <t>120001</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
         <is>
-          <t>650 TERRACE AVE</t>
+          <t>150 WAGARAW RD</t>
         </is>
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>HASBROUCK HEIGHTS</t>
-        </is>
-      </c>
-      <c r="M33" s="2" t="inlineStr">
-        <is>
-          <t>Drink Special</t>
-        </is>
-      </c>
-      <c r="N33" s="2" t="inlineStr">
-        <is>
-          <t>Table Tent</t>
-        </is>
-      </c>
+          <t>HAWTHORNE</t>
+        </is>
+      </c>
+      <c r="M33" s="2" t="n"/>
+      <c r="N33" s="2" t="n"/>
       <c r="O33" s="2" t="inlineStr">
         <is>
-          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+          <t>GREEN RIVER HONEY FINISHED BOURBON</t>
         </is>
       </c>
       <c r="P33" s="2" t="inlineStr">
@@ -3027,17 +3021,17 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>09/02/2026 09:10 AM</t>
+          <t>09/09/2026 04:48 PM</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>1.2</t>
+          <t>2.1</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>robin feldman</t>
+          <t>allison scott</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -3053,53 +3047,209 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
+          <t>Cocktail List Activation</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="n"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>BLACKJACK MULLIGAN'S PUBLIC HOUSE</t>
+        </is>
+      </c>
+      <c r="J34" s="2" t="inlineStr">
+        <is>
+          <t>15004</t>
+        </is>
+      </c>
+      <c r="K34" s="2" t="inlineStr">
+        <is>
+          <t>1145 MCBRIDE AVE</t>
+        </is>
+      </c>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>WOODLAND PARK</t>
+        </is>
+      </c>
+      <c r="M34" s="2" t="n"/>
+      <c r="N34" s="2" t="inlineStr">
+        <is>
+          <t>Menu</t>
+        </is>
+      </c>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>GREEN RIVER KENTUCKY STRAIGHT WHEATED BOURBON WHISKEY</t>
+        </is>
+      </c>
+      <c r="P34" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q34" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>1.1</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n"/>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
           <t>Feature Activation (on)</t>
         </is>
       </c>
-      <c r="H34" s="2" t="n">
+      <c r="H35" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I35" s="2" t="inlineStr">
         <is>
           <t>HILTON HASBRK HTS #50591</t>
         </is>
       </c>
-      <c r="J34" s="2" t="inlineStr">
+      <c r="J35" s="2" t="inlineStr">
         <is>
           <t>34018</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
+      <c r="K35" s="2" t="inlineStr">
         <is>
           <t>650 TERRACE AVE</t>
         </is>
       </c>
-      <c r="L34" s="2" t="inlineStr">
+      <c r="L35" s="2" t="inlineStr">
         <is>
           <t>HASBROUCK HEIGHTS</t>
         </is>
       </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="M35" s="2" t="inlineStr">
         <is>
           <t>Drink Special</t>
         </is>
       </c>
-      <c r="N34" s="2" t="inlineStr">
+      <c r="N35" s="2" t="inlineStr">
         <is>
           <t>Table Tent</t>
         </is>
       </c>
-      <c r="O34" s="2" t="inlineStr">
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COLLAB SERIES FOURSQUARE</t>
+        </is>
+      </c>
+      <c r="P35" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q35" s="3" t="inlineStr">
+        <is>
+          <t>Photo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>09/02/2026 09:10 AM</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>1.2</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>robin feldman</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t>Christopher McCrohan</t>
+        </is>
+      </c>
+      <c r="E36" s="2" t="n"/>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>Sales Rep</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Feature Activation (on)</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>HILTON HASBRK HTS #50591</t>
+        </is>
+      </c>
+      <c r="J36" s="2" t="inlineStr">
+        <is>
+          <t>34018</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>650 TERRACE AVE</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>HASBROUCK HEIGHTS</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>Drink Special</t>
+        </is>
+      </c>
+      <c r="N36" s="2" t="inlineStr">
+        <is>
+          <t>Table Tent</t>
+        </is>
+      </c>
+      <c r="O36" s="2" t="inlineStr">
         <is>
           <t>BARDSTOWN BOURBON COLLAB SERIES GOOSE ISLAND</t>
         </is>
       </c>
-      <c r="P34" s="2" t="inlineStr">
-        <is>
-          <t>BARDSTOWN BOURBON COMPANY</t>
-        </is>
-      </c>
-      <c r="Q34" s="3" t="inlineStr">
+      <c r="P36" s="2" t="inlineStr">
+        <is>
+          <t>BARDSTOWN BOURBON COMPANY</t>
+        </is>
+      </c>
+      <c r="Q36" s="3" t="inlineStr">
         <is>
           <t>Photo</t>
         </is>
@@ -3140,6 +3290,8 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q32" r:id="rId31"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Q36" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>